<commit_message>
fixed tests, code is formated
</commit_message>
<xml_diff>
--- a/tests/tests_data/transactions_test_excel.xlsx
+++ b/tests/tests_data/transactions_test_excel.xlsx
@@ -416,18 +416,18 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I1001"/>
-  <sheetFormatPr defaultColWidth="7.30078125" defaultRowHeight="19.9" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I1002"/>
+  <sheetFormatPr defaultColWidth="5.578125" defaultRowHeight="19.9" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="6.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.95"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="11.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="26.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="19.23"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="7.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="20.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.69"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="10" style="1" width="5.58"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -488,74 +488,74 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
+    <row r="3" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="n">
         <v>3598919</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D4" s="5" t="n">
         <v>29740</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H4" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
-        <v>593027</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>30368</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="A5" s="3" t="n">
+        <v>593027</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>30368</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3"/>
@@ -564,7 +564,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
-      <c r="G6" s="5"/>
+      <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
     </row>
@@ -575,7 +575,7 @@
       <c r="D7" s="5"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="G7" s="5"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
     </row>
@@ -597,7 +597,7 @@
       <c r="D9" s="5"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
-      <c r="G9" s="5"/>
+      <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
     </row>
@@ -619,7 +619,7 @@
       <c r="D11" s="5"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="G11" s="5"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
     </row>
@@ -641,7 +641,7 @@
       <c r="D13" s="5"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="5"/>
+      <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
     </row>
@@ -652,7 +652,7 @@
       <c r="D14" s="5"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
+      <c r="G14" s="5"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
     </row>
@@ -674,7 +674,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
-      <c r="G16" s="5"/>
+      <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
     </row>
@@ -685,7 +685,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
+      <c r="G17" s="5"/>
       <c r="H17" s="4"/>
       <c r="I17" s="4"/>
     </row>
@@ -762,7 +762,7 @@
       <c r="D24" s="5"/>
       <c r="E24" s="4"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="5"/>
+      <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="4"/>
     </row>
@@ -773,7 +773,7 @@
       <c r="D25" s="5"/>
       <c r="E25" s="4"/>
       <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="G25" s="5"/>
       <c r="H25" s="4"/>
       <c r="I25" s="4"/>
     </row>
@@ -839,7 +839,7 @@
       <c r="D31" s="5"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
-      <c r="G31" s="5"/>
+      <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
     </row>
@@ -861,7 +861,7 @@
       <c r="D33" s="5"/>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
+      <c r="G33" s="5"/>
       <c r="H33" s="4"/>
       <c r="I33" s="4"/>
     </row>
@@ -982,7 +982,7 @@
       <c r="D44" s="5"/>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
-      <c r="G44" s="5"/>
+      <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
     </row>
@@ -993,7 +993,7 @@
       <c r="D45" s="5"/>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
+      <c r="G45" s="5"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
     </row>
@@ -1004,7 +1004,7 @@
       <c r="D46" s="5"/>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
-      <c r="G46" s="5"/>
+      <c r="G46" s="4"/>
       <c r="H46" s="4"/>
       <c r="I46" s="4"/>
     </row>
@@ -1015,7 +1015,7 @@
       <c r="D47" s="5"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
+      <c r="G47" s="5"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4"/>
     </row>
@@ -1026,7 +1026,7 @@
       <c r="D48" s="5"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
-      <c r="G48" s="5"/>
+      <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4"/>
     </row>
@@ -1037,7 +1037,7 @@
       <c r="D49" s="5"/>
       <c r="E49" s="4"/>
       <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
+      <c r="G49" s="5"/>
       <c r="H49" s="4"/>
       <c r="I49" s="4"/>
     </row>
@@ -1048,7 +1048,7 @@
       <c r="D50" s="5"/>
       <c r="E50" s="4"/>
       <c r="F50" s="4"/>
-      <c r="G50" s="5"/>
+      <c r="G50" s="4"/>
       <c r="H50" s="4"/>
       <c r="I50" s="4"/>
     </row>
@@ -1059,7 +1059,7 @@
       <c r="D51" s="5"/>
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
+      <c r="G51" s="5"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
     </row>
@@ -1175,25 +1175,25 @@
     </row>
     <row r="62" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3"/>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
       <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
+      <c r="E62" s="4"/>
+      <c r="F62" s="4"/>
+      <c r="G62" s="4"/>
+      <c r="H62" s="4"/>
+      <c r="I62" s="4"/>
     </row>
     <row r="63" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="3"/>
-      <c r="B63" s="4"/>
-      <c r="C63" s="4"/>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
       <c r="D63" s="5"/>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
     </row>
     <row r="64" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3"/>
@@ -1235,7 +1235,7 @@
       <c r="D67" s="5"/>
       <c r="E67" s="4"/>
       <c r="F67" s="4"/>
-      <c r="G67" s="5"/>
+      <c r="G67" s="4"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4"/>
     </row>
@@ -1246,7 +1246,7 @@
       <c r="D68" s="5"/>
       <c r="E68" s="4"/>
       <c r="F68" s="4"/>
-      <c r="G68" s="4"/>
+      <c r="G68" s="5"/>
       <c r="H68" s="4"/>
       <c r="I68" s="4"/>
     </row>
@@ -1257,7 +1257,7 @@
       <c r="D69" s="5"/>
       <c r="E69" s="4"/>
       <c r="F69" s="4"/>
-      <c r="G69" s="5"/>
+      <c r="G69" s="4"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4"/>
     </row>
@@ -1268,7 +1268,7 @@
       <c r="D70" s="5"/>
       <c r="E70" s="4"/>
       <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
+      <c r="G70" s="5"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4"/>
     </row>
@@ -1422,7 +1422,7 @@
       <c r="D84" s="5"/>
       <c r="E84" s="4"/>
       <c r="F84" s="4"/>
-      <c r="G84" s="5"/>
+      <c r="G84" s="4"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4"/>
     </row>
@@ -1433,7 +1433,7 @@
       <c r="D85" s="5"/>
       <c r="E85" s="4"/>
       <c r="F85" s="4"/>
-      <c r="G85" s="4"/>
+      <c r="G85" s="5"/>
       <c r="H85" s="4"/>
       <c r="I85" s="4"/>
     </row>
@@ -1444,7 +1444,7 @@
       <c r="D86" s="5"/>
       <c r="E86" s="4"/>
       <c r="F86" s="4"/>
-      <c r="G86" s="5"/>
+      <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4"/>
     </row>
@@ -1455,7 +1455,7 @@
       <c r="D87" s="5"/>
       <c r="E87" s="4"/>
       <c r="F87" s="4"/>
-      <c r="G87" s="4"/>
+      <c r="G87" s="5"/>
       <c r="H87" s="4"/>
       <c r="I87" s="4"/>
     </row>
@@ -1587,7 +1587,7 @@
       <c r="D99" s="5"/>
       <c r="E99" s="4"/>
       <c r="F99" s="4"/>
-      <c r="G99" s="5"/>
+      <c r="G99" s="4"/>
       <c r="H99" s="4"/>
       <c r="I99" s="4"/>
     </row>
@@ -1598,7 +1598,7 @@
       <c r="D100" s="5"/>
       <c r="E100" s="4"/>
       <c r="F100" s="4"/>
-      <c r="G100" s="4"/>
+      <c r="G100" s="5"/>
       <c r="H100" s="4"/>
       <c r="I100" s="4"/>
     </row>
@@ -1631,7 +1631,7 @@
       <c r="D103" s="5"/>
       <c r="E103" s="4"/>
       <c r="F103" s="4"/>
-      <c r="G103" s="5"/>
+      <c r="G103" s="4"/>
       <c r="H103" s="4"/>
       <c r="I103" s="4"/>
     </row>
@@ -1664,7 +1664,7 @@
       <c r="D106" s="5"/>
       <c r="E106" s="4"/>
       <c r="F106" s="4"/>
-      <c r="G106" s="4"/>
+      <c r="G106" s="5"/>
       <c r="H106" s="4"/>
       <c r="I106" s="4"/>
     </row>
@@ -1796,7 +1796,7 @@
       <c r="D118" s="5"/>
       <c r="E118" s="4"/>
       <c r="F118" s="4"/>
-      <c r="G118" s="5"/>
+      <c r="G118" s="4"/>
       <c r="H118" s="4"/>
       <c r="I118" s="4"/>
     </row>
@@ -1807,7 +1807,7 @@
       <c r="D119" s="5"/>
       <c r="E119" s="4"/>
       <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
+      <c r="G119" s="5"/>
       <c r="H119" s="4"/>
       <c r="I119" s="4"/>
     </row>
@@ -1862,7 +1862,7 @@
       <c r="D124" s="5"/>
       <c r="E124" s="4"/>
       <c r="F124" s="4"/>
-      <c r="G124" s="5"/>
+      <c r="G124" s="4"/>
       <c r="H124" s="4"/>
       <c r="I124" s="4"/>
     </row>
@@ -1884,7 +1884,7 @@
       <c r="D126" s="5"/>
       <c r="E126" s="4"/>
       <c r="F126" s="4"/>
-      <c r="G126" s="4"/>
+      <c r="G126" s="5"/>
       <c r="H126" s="4"/>
       <c r="I126" s="4"/>
     </row>
@@ -1906,7 +1906,7 @@
       <c r="D128" s="5"/>
       <c r="E128" s="4"/>
       <c r="F128" s="4"/>
-      <c r="G128" s="5"/>
+      <c r="G128" s="4"/>
       <c r="H128" s="4"/>
       <c r="I128" s="4"/>
     </row>
@@ -1917,7 +1917,7 @@
       <c r="D129" s="5"/>
       <c r="E129" s="4"/>
       <c r="F129" s="4"/>
-      <c r="G129" s="4"/>
+      <c r="G129" s="5"/>
       <c r="H129" s="4"/>
       <c r="I129" s="4"/>
     </row>
@@ -1961,7 +1961,7 @@
       <c r="D133" s="5"/>
       <c r="E133" s="4"/>
       <c r="F133" s="4"/>
-      <c r="G133" s="5"/>
+      <c r="G133" s="4"/>
       <c r="H133" s="4"/>
       <c r="I133" s="4"/>
     </row>
@@ -1983,7 +1983,7 @@
       <c r="D135" s="5"/>
       <c r="E135" s="4"/>
       <c r="F135" s="4"/>
-      <c r="G135" s="4"/>
+      <c r="G135" s="5"/>
       <c r="H135" s="4"/>
       <c r="I135" s="4"/>
     </row>
@@ -2016,7 +2016,7 @@
       <c r="D138" s="5"/>
       <c r="E138" s="4"/>
       <c r="F138" s="4"/>
-      <c r="G138" s="5"/>
+      <c r="G138" s="4"/>
       <c r="H138" s="4"/>
       <c r="I138" s="4"/>
     </row>
@@ -2038,7 +2038,7 @@
       <c r="D140" s="5"/>
       <c r="E140" s="4"/>
       <c r="F140" s="4"/>
-      <c r="G140" s="4"/>
+      <c r="G140" s="5"/>
       <c r="H140" s="4"/>
       <c r="I140" s="4"/>
     </row>
@@ -2093,7 +2093,7 @@
       <c r="D145" s="5"/>
       <c r="E145" s="4"/>
       <c r="F145" s="4"/>
-      <c r="G145" s="5"/>
+      <c r="G145" s="4"/>
       <c r="H145" s="4"/>
       <c r="I145" s="4"/>
     </row>
@@ -2104,7 +2104,7 @@
       <c r="D146" s="5"/>
       <c r="E146" s="4"/>
       <c r="F146" s="4"/>
-      <c r="G146" s="4"/>
+      <c r="G146" s="5"/>
       <c r="H146" s="4"/>
       <c r="I146" s="4"/>
     </row>
@@ -2258,7 +2258,7 @@
       <c r="D160" s="5"/>
       <c r="E160" s="4"/>
       <c r="F160" s="4"/>
-      <c r="G160" s="5"/>
+      <c r="G160" s="4"/>
       <c r="H160" s="4"/>
       <c r="I160" s="4"/>
     </row>
@@ -2269,7 +2269,7 @@
       <c r="D161" s="5"/>
       <c r="E161" s="4"/>
       <c r="F161" s="4"/>
-      <c r="G161" s="4"/>
+      <c r="G161" s="5"/>
       <c r="H161" s="4"/>
       <c r="I161" s="4"/>
     </row>
@@ -2346,7 +2346,7 @@
       <c r="D168" s="5"/>
       <c r="E168" s="4"/>
       <c r="F168" s="4"/>
-      <c r="G168" s="5"/>
+      <c r="G168" s="4"/>
       <c r="H168" s="4"/>
       <c r="I168" s="4"/>
     </row>
@@ -2357,7 +2357,7 @@
       <c r="D169" s="5"/>
       <c r="E169" s="4"/>
       <c r="F169" s="4"/>
-      <c r="G169" s="4"/>
+      <c r="G169" s="5"/>
       <c r="H169" s="4"/>
       <c r="I169" s="4"/>
     </row>
@@ -2434,7 +2434,7 @@
       <c r="D176" s="5"/>
       <c r="E176" s="4"/>
       <c r="F176" s="4"/>
-      <c r="G176" s="5"/>
+      <c r="G176" s="4"/>
       <c r="H176" s="4"/>
       <c r="I176" s="4"/>
     </row>
@@ -2445,7 +2445,7 @@
       <c r="D177" s="5"/>
       <c r="E177" s="4"/>
       <c r="F177" s="4"/>
-      <c r="G177" s="4"/>
+      <c r="G177" s="5"/>
       <c r="H177" s="4"/>
       <c r="I177" s="4"/>
     </row>
@@ -2478,7 +2478,7 @@
       <c r="D180" s="5"/>
       <c r="E180" s="4"/>
       <c r="F180" s="4"/>
-      <c r="G180" s="5"/>
+      <c r="G180" s="4"/>
       <c r="H180" s="4"/>
       <c r="I180" s="4"/>
     </row>
@@ -2489,7 +2489,7 @@
       <c r="D181" s="5"/>
       <c r="E181" s="4"/>
       <c r="F181" s="4"/>
-      <c r="G181" s="4"/>
+      <c r="G181" s="5"/>
       <c r="H181" s="4"/>
       <c r="I181" s="4"/>
     </row>
@@ -2500,7 +2500,7 @@
       <c r="D182" s="5"/>
       <c r="E182" s="4"/>
       <c r="F182" s="4"/>
-      <c r="G182" s="5"/>
+      <c r="G182" s="4"/>
       <c r="H182" s="4"/>
       <c r="I182" s="4"/>
     </row>
@@ -2511,7 +2511,7 @@
       <c r="D183" s="5"/>
       <c r="E183" s="4"/>
       <c r="F183" s="4"/>
-      <c r="G183" s="4"/>
+      <c r="G183" s="5"/>
       <c r="H183" s="4"/>
       <c r="I183" s="4"/>
     </row>
@@ -2599,7 +2599,7 @@
       <c r="D191" s="5"/>
       <c r="E191" s="4"/>
       <c r="F191" s="4"/>
-      <c r="G191" s="5"/>
+      <c r="G191" s="4"/>
       <c r="H191" s="4"/>
       <c r="I191" s="4"/>
     </row>
@@ -2621,7 +2621,7 @@
       <c r="D193" s="5"/>
       <c r="E193" s="4"/>
       <c r="F193" s="4"/>
-      <c r="G193" s="4"/>
+      <c r="G193" s="5"/>
       <c r="H193" s="4"/>
       <c r="I193" s="4"/>
     </row>
@@ -2665,7 +2665,7 @@
       <c r="D197" s="5"/>
       <c r="E197" s="4"/>
       <c r="F197" s="4"/>
-      <c r="G197" s="5"/>
+      <c r="G197" s="4"/>
       <c r="H197" s="4"/>
       <c r="I197" s="4"/>
     </row>
@@ -2676,7 +2676,7 @@
       <c r="D198" s="5"/>
       <c r="E198" s="4"/>
       <c r="F198" s="4"/>
-      <c r="G198" s="4"/>
+      <c r="G198" s="5"/>
       <c r="H198" s="4"/>
       <c r="I198" s="4"/>
     </row>
@@ -2753,7 +2753,7 @@
       <c r="D205" s="5"/>
       <c r="E205" s="4"/>
       <c r="F205" s="4"/>
-      <c r="G205" s="5"/>
+      <c r="G205" s="4"/>
       <c r="H205" s="4"/>
       <c r="I205" s="4"/>
     </row>
@@ -2764,7 +2764,7 @@
       <c r="D206" s="5"/>
       <c r="E206" s="4"/>
       <c r="F206" s="4"/>
-      <c r="G206" s="4"/>
+      <c r="G206" s="5"/>
       <c r="H206" s="4"/>
       <c r="I206" s="4"/>
     </row>
@@ -2797,7 +2797,7 @@
       <c r="D209" s="5"/>
       <c r="E209" s="4"/>
       <c r="F209" s="4"/>
-      <c r="G209" s="5"/>
+      <c r="G209" s="4"/>
       <c r="H209" s="4"/>
       <c r="I209" s="4"/>
     </row>
@@ -2808,7 +2808,7 @@
       <c r="D210" s="5"/>
       <c r="E210" s="4"/>
       <c r="F210" s="4"/>
-      <c r="G210" s="4"/>
+      <c r="G210" s="5"/>
       <c r="H210" s="4"/>
       <c r="I210" s="4"/>
     </row>
@@ -2896,7 +2896,7 @@
       <c r="D218" s="5"/>
       <c r="E218" s="4"/>
       <c r="F218" s="4"/>
-      <c r="G218" s="5"/>
+      <c r="G218" s="4"/>
       <c r="H218" s="4"/>
       <c r="I218" s="4"/>
     </row>
@@ -2907,7 +2907,7 @@
       <c r="D219" s="5"/>
       <c r="E219" s="4"/>
       <c r="F219" s="4"/>
-      <c r="G219" s="4"/>
+      <c r="G219" s="5"/>
       <c r="H219" s="4"/>
       <c r="I219" s="4"/>
     </row>
@@ -2951,7 +2951,7 @@
       <c r="D223" s="5"/>
       <c r="E223" s="4"/>
       <c r="F223" s="4"/>
-      <c r="G223" s="5"/>
+      <c r="G223" s="4"/>
       <c r="H223" s="4"/>
       <c r="I223" s="4"/>
     </row>
@@ -2962,7 +2962,7 @@
       <c r="D224" s="5"/>
       <c r="E224" s="4"/>
       <c r="F224" s="4"/>
-      <c r="G224" s="4"/>
+      <c r="G224" s="5"/>
       <c r="H224" s="4"/>
       <c r="I224" s="4"/>
     </row>
@@ -3006,7 +3006,7 @@
       <c r="D228" s="5"/>
       <c r="E228" s="4"/>
       <c r="F228" s="4"/>
-      <c r="G228" s="5"/>
+      <c r="G228" s="4"/>
       <c r="H228" s="4"/>
       <c r="I228" s="4"/>
     </row>
@@ -3039,7 +3039,7 @@
       <c r="D231" s="5"/>
       <c r="E231" s="4"/>
       <c r="F231" s="4"/>
-      <c r="G231" s="4"/>
+      <c r="G231" s="5"/>
       <c r="H231" s="4"/>
       <c r="I231" s="4"/>
     </row>
@@ -3072,7 +3072,7 @@
       <c r="D234" s="5"/>
       <c r="E234" s="4"/>
       <c r="F234" s="4"/>
-      <c r="G234" s="5"/>
+      <c r="G234" s="4"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
     </row>
@@ -3083,7 +3083,7 @@
       <c r="D235" s="5"/>
       <c r="E235" s="4"/>
       <c r="F235" s="4"/>
-      <c r="G235" s="4"/>
+      <c r="G235" s="5"/>
       <c r="H235" s="4"/>
       <c r="I235" s="4"/>
     </row>
@@ -3116,7 +3116,7 @@
       <c r="D238" s="5"/>
       <c r="E238" s="4"/>
       <c r="F238" s="4"/>
-      <c r="G238" s="5"/>
+      <c r="G238" s="4"/>
       <c r="H238" s="4"/>
       <c r="I238" s="4"/>
     </row>
@@ -3127,7 +3127,7 @@
       <c r="D239" s="5"/>
       <c r="E239" s="4"/>
       <c r="F239" s="4"/>
-      <c r="G239" s="4"/>
+      <c r="G239" s="5"/>
       <c r="H239" s="4"/>
       <c r="I239" s="4"/>
     </row>
@@ -3138,7 +3138,7 @@
       <c r="D240" s="5"/>
       <c r="E240" s="4"/>
       <c r="F240" s="4"/>
-      <c r="G240" s="5"/>
+      <c r="G240" s="4"/>
       <c r="H240" s="4"/>
       <c r="I240" s="4"/>
     </row>
@@ -3149,7 +3149,7 @@
       <c r="D241" s="5"/>
       <c r="E241" s="4"/>
       <c r="F241" s="4"/>
-      <c r="G241" s="4"/>
+      <c r="G241" s="5"/>
       <c r="H241" s="4"/>
       <c r="I241" s="4"/>
     </row>
@@ -3160,7 +3160,7 @@
       <c r="D242" s="5"/>
       <c r="E242" s="4"/>
       <c r="F242" s="4"/>
-      <c r="G242" s="5"/>
+      <c r="G242" s="4"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
     </row>
@@ -3171,7 +3171,7 @@
       <c r="D243" s="5"/>
       <c r="E243" s="4"/>
       <c r="F243" s="4"/>
-      <c r="G243" s="4"/>
+      <c r="G243" s="5"/>
       <c r="H243" s="4"/>
       <c r="I243" s="4"/>
     </row>
@@ -3204,7 +3204,7 @@
       <c r="D246" s="5"/>
       <c r="E246" s="4"/>
       <c r="F246" s="4"/>
-      <c r="G246" s="5"/>
+      <c r="G246" s="4"/>
       <c r="H246" s="4"/>
       <c r="I246" s="4"/>
     </row>
@@ -3215,7 +3215,7 @@
       <c r="D247" s="5"/>
       <c r="E247" s="4"/>
       <c r="F247" s="4"/>
-      <c r="G247" s="4"/>
+      <c r="G247" s="5"/>
       <c r="H247" s="4"/>
       <c r="I247" s="4"/>
     </row>
@@ -3226,7 +3226,7 @@
       <c r="D248" s="5"/>
       <c r="E248" s="4"/>
       <c r="F248" s="4"/>
-      <c r="G248" s="5"/>
+      <c r="G248" s="4"/>
       <c r="H248" s="4"/>
       <c r="I248" s="4"/>
     </row>
@@ -3259,7 +3259,7 @@
       <c r="D251" s="5"/>
       <c r="E251" s="4"/>
       <c r="F251" s="4"/>
-      <c r="G251" s="4"/>
+      <c r="G251" s="5"/>
       <c r="H251" s="4"/>
       <c r="I251" s="4"/>
     </row>
@@ -3281,7 +3281,7 @@
       <c r="D253" s="5"/>
       <c r="E253" s="4"/>
       <c r="F253" s="4"/>
-      <c r="G253" s="5"/>
+      <c r="G253" s="4"/>
       <c r="H253" s="4"/>
       <c r="I253" s="4"/>
     </row>
@@ -3292,7 +3292,7 @@
       <c r="D254" s="5"/>
       <c r="E254" s="4"/>
       <c r="F254" s="4"/>
-      <c r="G254" s="4"/>
+      <c r="G254" s="5"/>
       <c r="H254" s="4"/>
       <c r="I254" s="4"/>
     </row>
@@ -3314,7 +3314,7 @@
       <c r="D256" s="5"/>
       <c r="E256" s="4"/>
       <c r="F256" s="4"/>
-      <c r="G256" s="5"/>
+      <c r="G256" s="4"/>
       <c r="H256" s="4"/>
       <c r="I256" s="4"/>
     </row>
@@ -3325,7 +3325,7 @@
       <c r="D257" s="5"/>
       <c r="E257" s="4"/>
       <c r="F257" s="4"/>
-      <c r="G257" s="4"/>
+      <c r="G257" s="5"/>
       <c r="H257" s="4"/>
       <c r="I257" s="4"/>
     </row>
@@ -3336,7 +3336,7 @@
       <c r="D258" s="5"/>
       <c r="E258" s="4"/>
       <c r="F258" s="4"/>
-      <c r="G258" s="5"/>
+      <c r="G258" s="4"/>
       <c r="H258" s="4"/>
       <c r="I258" s="4"/>
     </row>
@@ -3347,7 +3347,7 @@
       <c r="D259" s="5"/>
       <c r="E259" s="4"/>
       <c r="F259" s="4"/>
-      <c r="G259" s="4"/>
+      <c r="G259" s="5"/>
       <c r="H259" s="4"/>
       <c r="I259" s="4"/>
     </row>
@@ -3391,7 +3391,7 @@
       <c r="D263" s="5"/>
       <c r="E263" s="4"/>
       <c r="F263" s="4"/>
-      <c r="G263" s="5"/>
+      <c r="G263" s="4"/>
       <c r="H263" s="4"/>
       <c r="I263" s="4"/>
     </row>
@@ -3402,7 +3402,7 @@
       <c r="D264" s="5"/>
       <c r="E264" s="4"/>
       <c r="F264" s="4"/>
-      <c r="G264" s="4"/>
+      <c r="G264" s="5"/>
       <c r="H264" s="4"/>
       <c r="I264" s="4"/>
     </row>
@@ -3545,7 +3545,7 @@
       <c r="D277" s="5"/>
       <c r="E277" s="4"/>
       <c r="F277" s="4"/>
-      <c r="G277" s="5"/>
+      <c r="G277" s="4"/>
       <c r="H277" s="4"/>
       <c r="I277" s="4"/>
     </row>
@@ -3556,7 +3556,7 @@
       <c r="D278" s="5"/>
       <c r="E278" s="4"/>
       <c r="F278" s="4"/>
-      <c r="G278" s="4"/>
+      <c r="G278" s="5"/>
       <c r="H278" s="4"/>
       <c r="I278" s="4"/>
     </row>
@@ -3567,7 +3567,7 @@
       <c r="D279" s="5"/>
       <c r="E279" s="4"/>
       <c r="F279" s="4"/>
-      <c r="G279" s="5"/>
+      <c r="G279" s="4"/>
       <c r="H279" s="4"/>
       <c r="I279" s="4"/>
     </row>
@@ -3578,7 +3578,7 @@
       <c r="D280" s="5"/>
       <c r="E280" s="4"/>
       <c r="F280" s="4"/>
-      <c r="G280" s="4"/>
+      <c r="G280" s="5"/>
       <c r="H280" s="4"/>
       <c r="I280" s="4"/>
     </row>
@@ -3633,7 +3633,7 @@
       <c r="D285" s="5"/>
       <c r="E285" s="4"/>
       <c r="F285" s="4"/>
-      <c r="G285" s="5"/>
+      <c r="G285" s="4"/>
       <c r="H285" s="4"/>
       <c r="I285" s="4"/>
     </row>
@@ -3644,7 +3644,7 @@
       <c r="D286" s="5"/>
       <c r="E286" s="4"/>
       <c r="F286" s="4"/>
-      <c r="G286" s="4"/>
+      <c r="G286" s="5"/>
       <c r="H286" s="4"/>
       <c r="I286" s="4"/>
     </row>
@@ -3677,7 +3677,7 @@
       <c r="D289" s="5"/>
       <c r="E289" s="4"/>
       <c r="F289" s="4"/>
-      <c r="G289" s="5"/>
+      <c r="G289" s="4"/>
       <c r="H289" s="4"/>
       <c r="I289" s="4"/>
     </row>
@@ -3688,7 +3688,7 @@
       <c r="D290" s="5"/>
       <c r="E290" s="4"/>
       <c r="F290" s="4"/>
-      <c r="G290" s="4"/>
+      <c r="G290" s="5"/>
       <c r="H290" s="4"/>
       <c r="I290" s="4"/>
     </row>
@@ -3699,7 +3699,7 @@
       <c r="D291" s="5"/>
       <c r="E291" s="4"/>
       <c r="F291" s="4"/>
-      <c r="G291" s="5"/>
+      <c r="G291" s="4"/>
       <c r="H291" s="4"/>
       <c r="I291" s="4"/>
     </row>
@@ -3710,7 +3710,7 @@
       <c r="D292" s="5"/>
       <c r="E292" s="4"/>
       <c r="F292" s="4"/>
-      <c r="G292" s="4"/>
+      <c r="G292" s="5"/>
       <c r="H292" s="4"/>
       <c r="I292" s="4"/>
     </row>
@@ -3754,7 +3754,7 @@
       <c r="D296" s="5"/>
       <c r="E296" s="4"/>
       <c r="F296" s="4"/>
-      <c r="G296" s="5"/>
+      <c r="G296" s="4"/>
       <c r="H296" s="4"/>
       <c r="I296" s="4"/>
     </row>
@@ -3765,7 +3765,7 @@
       <c r="D297" s="5"/>
       <c r="E297" s="4"/>
       <c r="F297" s="4"/>
-      <c r="G297" s="4"/>
+      <c r="G297" s="5"/>
       <c r="H297" s="4"/>
       <c r="I297" s="4"/>
     </row>
@@ -3941,7 +3941,7 @@
       <c r="D313" s="5"/>
       <c r="E313" s="4"/>
       <c r="F313" s="4"/>
-      <c r="G313" s="5"/>
+      <c r="G313" s="4"/>
       <c r="H313" s="4"/>
       <c r="I313" s="4"/>
     </row>
@@ -3952,7 +3952,7 @@
       <c r="D314" s="5"/>
       <c r="E314" s="4"/>
       <c r="F314" s="4"/>
-      <c r="G314" s="4"/>
+      <c r="G314" s="5"/>
       <c r="H314" s="4"/>
       <c r="I314" s="4"/>
     </row>
@@ -4007,7 +4007,7 @@
       <c r="D319" s="5"/>
       <c r="E319" s="4"/>
       <c r="F319" s="4"/>
-      <c r="G319" s="5"/>
+      <c r="G319" s="4"/>
       <c r="H319" s="4"/>
       <c r="I319" s="4"/>
     </row>
@@ -4018,7 +4018,7 @@
       <c r="D320" s="5"/>
       <c r="E320" s="4"/>
       <c r="F320" s="4"/>
-      <c r="G320" s="4"/>
+      <c r="G320" s="5"/>
       <c r="H320" s="4"/>
       <c r="I320" s="4"/>
     </row>
@@ -4029,7 +4029,7 @@
       <c r="D321" s="5"/>
       <c r="E321" s="4"/>
       <c r="F321" s="4"/>
-      <c r="G321" s="5"/>
+      <c r="G321" s="4"/>
       <c r="H321" s="4"/>
       <c r="I321" s="4"/>
     </row>
@@ -4040,7 +4040,7 @@
       <c r="D322" s="5"/>
       <c r="E322" s="4"/>
       <c r="F322" s="4"/>
-      <c r="G322" s="4"/>
+      <c r="G322" s="5"/>
       <c r="H322" s="4"/>
       <c r="I322" s="4"/>
     </row>
@@ -4062,7 +4062,7 @@
       <c r="D324" s="5"/>
       <c r="E324" s="4"/>
       <c r="F324" s="4"/>
-      <c r="G324" s="5"/>
+      <c r="G324" s="4"/>
       <c r="H324" s="4"/>
       <c r="I324" s="4"/>
     </row>
@@ -4073,7 +4073,7 @@
       <c r="D325" s="5"/>
       <c r="E325" s="4"/>
       <c r="F325" s="4"/>
-      <c r="G325" s="4"/>
+      <c r="G325" s="5"/>
       <c r="H325" s="4"/>
       <c r="I325" s="4"/>
     </row>
@@ -4084,7 +4084,7 @@
       <c r="D326" s="5"/>
       <c r="E326" s="4"/>
       <c r="F326" s="4"/>
-      <c r="G326" s="5"/>
+      <c r="G326" s="4"/>
       <c r="H326" s="4"/>
       <c r="I326" s="4"/>
     </row>
@@ -4095,7 +4095,7 @@
       <c r="D327" s="5"/>
       <c r="E327" s="4"/>
       <c r="F327" s="4"/>
-      <c r="G327" s="4"/>
+      <c r="G327" s="5"/>
       <c r="H327" s="4"/>
       <c r="I327" s="4"/>
     </row>
@@ -4150,7 +4150,7 @@
       <c r="D332" s="5"/>
       <c r="E332" s="4"/>
       <c r="F332" s="4"/>
-      <c r="G332" s="5"/>
+      <c r="G332" s="4"/>
       <c r="H332" s="4"/>
       <c r="I332" s="4"/>
     </row>
@@ -4172,7 +4172,7 @@
       <c r="D334" s="5"/>
       <c r="E334" s="4"/>
       <c r="F334" s="4"/>
-      <c r="G334" s="4"/>
+      <c r="G334" s="5"/>
       <c r="H334" s="4"/>
       <c r="I334" s="4"/>
     </row>
@@ -4227,7 +4227,7 @@
       <c r="D339" s="5"/>
       <c r="E339" s="4"/>
       <c r="F339" s="4"/>
-      <c r="G339" s="5"/>
+      <c r="G339" s="4"/>
       <c r="H339" s="4"/>
       <c r="I339" s="4"/>
     </row>
@@ -4260,7 +4260,7 @@
       <c r="D342" s="5"/>
       <c r="E342" s="4"/>
       <c r="F342" s="4"/>
-      <c r="G342" s="4"/>
+      <c r="G342" s="5"/>
       <c r="H342" s="4"/>
       <c r="I342" s="4"/>
     </row>
@@ -4271,7 +4271,7 @@
       <c r="D343" s="5"/>
       <c r="E343" s="4"/>
       <c r="F343" s="4"/>
-      <c r="G343" s="5"/>
+      <c r="G343" s="4"/>
       <c r="H343" s="4"/>
       <c r="I343" s="4"/>
     </row>
@@ -4293,7 +4293,7 @@
       <c r="D345" s="5"/>
       <c r="E345" s="4"/>
       <c r="F345" s="4"/>
-      <c r="G345" s="4"/>
+      <c r="G345" s="5"/>
       <c r="H345" s="4"/>
       <c r="I345" s="4"/>
     </row>
@@ -4414,7 +4414,7 @@
       <c r="D356" s="5"/>
       <c r="E356" s="4"/>
       <c r="F356" s="4"/>
-      <c r="G356" s="5"/>
+      <c r="G356" s="4"/>
       <c r="H356" s="4"/>
       <c r="I356" s="4"/>
     </row>
@@ -4425,7 +4425,7 @@
       <c r="D357" s="5"/>
       <c r="E357" s="4"/>
       <c r="F357" s="4"/>
-      <c r="G357" s="4"/>
+      <c r="G357" s="5"/>
       <c r="H357" s="4"/>
       <c r="I357" s="4"/>
     </row>
@@ -4436,7 +4436,7 @@
       <c r="D358" s="5"/>
       <c r="E358" s="4"/>
       <c r="F358" s="4"/>
-      <c r="G358" s="5"/>
+      <c r="G358" s="4"/>
       <c r="H358" s="4"/>
       <c r="I358" s="4"/>
     </row>
@@ -4458,7 +4458,7 @@
       <c r="D360" s="5"/>
       <c r="E360" s="4"/>
       <c r="F360" s="4"/>
-      <c r="G360" s="4"/>
+      <c r="G360" s="5"/>
       <c r="H360" s="4"/>
       <c r="I360" s="4"/>
     </row>
@@ -4502,7 +4502,7 @@
       <c r="D364" s="5"/>
       <c r="E364" s="4"/>
       <c r="F364" s="4"/>
-      <c r="G364" s="5"/>
+      <c r="G364" s="4"/>
       <c r="H364" s="4"/>
       <c r="I364" s="4"/>
     </row>
@@ -4524,7 +4524,7 @@
       <c r="D366" s="5"/>
       <c r="E366" s="4"/>
       <c r="F366" s="4"/>
-      <c r="G366" s="4"/>
+      <c r="G366" s="5"/>
       <c r="H366" s="4"/>
       <c r="I366" s="4"/>
     </row>
@@ -4579,7 +4579,7 @@
       <c r="D371" s="5"/>
       <c r="E371" s="4"/>
       <c r="F371" s="4"/>
-      <c r="G371" s="5"/>
+      <c r="G371" s="4"/>
       <c r="H371" s="4"/>
       <c r="I371" s="4"/>
     </row>
@@ -4590,7 +4590,7 @@
       <c r="D372" s="5"/>
       <c r="E372" s="4"/>
       <c r="F372" s="4"/>
-      <c r="G372" s="4"/>
+      <c r="G372" s="5"/>
       <c r="H372" s="4"/>
       <c r="I372" s="4"/>
     </row>
@@ -4667,7 +4667,7 @@
       <c r="D379" s="5"/>
       <c r="E379" s="4"/>
       <c r="F379" s="4"/>
-      <c r="G379" s="5"/>
+      <c r="G379" s="4"/>
       <c r="H379" s="4"/>
       <c r="I379" s="4"/>
     </row>
@@ -4678,7 +4678,7 @@
       <c r="D380" s="5"/>
       <c r="E380" s="4"/>
       <c r="F380" s="4"/>
-      <c r="G380" s="4"/>
+      <c r="G380" s="5"/>
       <c r="H380" s="4"/>
       <c r="I380" s="4"/>
     </row>
@@ -4733,7 +4733,7 @@
       <c r="D385" s="5"/>
       <c r="E385" s="4"/>
       <c r="F385" s="4"/>
-      <c r="G385" s="5"/>
+      <c r="G385" s="4"/>
       <c r="H385" s="4"/>
       <c r="I385" s="4"/>
     </row>
@@ -4744,7 +4744,7 @@
       <c r="D386" s="5"/>
       <c r="E386" s="4"/>
       <c r="F386" s="4"/>
-      <c r="G386" s="4"/>
+      <c r="G386" s="5"/>
       <c r="H386" s="4"/>
       <c r="I386" s="4"/>
     </row>
@@ -4777,7 +4777,7 @@
       <c r="D389" s="5"/>
       <c r="E389" s="4"/>
       <c r="F389" s="4"/>
-      <c r="G389" s="5"/>
+      <c r="G389" s="4"/>
       <c r="H389" s="4"/>
       <c r="I389" s="4"/>
     </row>
@@ -4788,7 +4788,7 @@
       <c r="D390" s="5"/>
       <c r="E390" s="4"/>
       <c r="F390" s="4"/>
-      <c r="G390" s="4"/>
+      <c r="G390" s="5"/>
       <c r="H390" s="4"/>
       <c r="I390" s="4"/>
     </row>
@@ -4821,7 +4821,7 @@
       <c r="D393" s="5"/>
       <c r="E393" s="4"/>
       <c r="F393" s="4"/>
-      <c r="G393" s="5"/>
+      <c r="G393" s="4"/>
       <c r="H393" s="4"/>
       <c r="I393" s="4"/>
     </row>
@@ -4843,7 +4843,7 @@
       <c r="D395" s="5"/>
       <c r="E395" s="4"/>
       <c r="F395" s="4"/>
-      <c r="G395" s="4"/>
+      <c r="G395" s="5"/>
       <c r="H395" s="4"/>
       <c r="I395" s="4"/>
     </row>
@@ -4931,7 +4931,7 @@
       <c r="D403" s="5"/>
       <c r="E403" s="4"/>
       <c r="F403" s="4"/>
-      <c r="G403" s="5"/>
+      <c r="G403" s="4"/>
       <c r="H403" s="4"/>
       <c r="I403" s="4"/>
     </row>
@@ -4942,7 +4942,7 @@
       <c r="D404" s="5"/>
       <c r="E404" s="4"/>
       <c r="F404" s="4"/>
-      <c r="G404" s="4"/>
+      <c r="G404" s="5"/>
       <c r="H404" s="4"/>
       <c r="I404" s="4"/>
     </row>
@@ -4975,7 +4975,7 @@
       <c r="D407" s="5"/>
       <c r="E407" s="4"/>
       <c r="F407" s="4"/>
-      <c r="G407" s="5"/>
+      <c r="G407" s="4"/>
       <c r="H407" s="4"/>
       <c r="I407" s="4"/>
     </row>
@@ -4986,7 +4986,7 @@
       <c r="D408" s="5"/>
       <c r="E408" s="4"/>
       <c r="F408" s="4"/>
-      <c r="G408" s="4"/>
+      <c r="G408" s="5"/>
       <c r="H408" s="4"/>
       <c r="I408" s="4"/>
     </row>
@@ -5019,7 +5019,7 @@
       <c r="D411" s="5"/>
       <c r="E411" s="4"/>
       <c r="F411" s="4"/>
-      <c r="G411" s="5"/>
+      <c r="G411" s="4"/>
       <c r="H411" s="4"/>
       <c r="I411" s="4"/>
     </row>
@@ -5030,7 +5030,7 @@
       <c r="D412" s="5"/>
       <c r="E412" s="4"/>
       <c r="F412" s="4"/>
-      <c r="G412" s="4"/>
+      <c r="G412" s="5"/>
       <c r="H412" s="4"/>
       <c r="I412" s="4"/>
     </row>
@@ -5140,7 +5140,7 @@
       <c r="D422" s="5"/>
       <c r="E422" s="4"/>
       <c r="F422" s="4"/>
-      <c r="G422" s="5"/>
+      <c r="G422" s="4"/>
       <c r="H422" s="4"/>
       <c r="I422" s="4"/>
     </row>
@@ -5151,7 +5151,7 @@
       <c r="D423" s="5"/>
       <c r="E423" s="4"/>
       <c r="F423" s="4"/>
-      <c r="G423" s="4"/>
+      <c r="G423" s="5"/>
       <c r="H423" s="4"/>
       <c r="I423" s="4"/>
     </row>
@@ -5217,7 +5217,7 @@
       <c r="D429" s="5"/>
       <c r="E429" s="4"/>
       <c r="F429" s="4"/>
-      <c r="G429" s="5"/>
+      <c r="G429" s="4"/>
       <c r="H429" s="4"/>
       <c r="I429" s="4"/>
     </row>
@@ -5228,7 +5228,7 @@
       <c r="D430" s="5"/>
       <c r="E430" s="4"/>
       <c r="F430" s="4"/>
-      <c r="G430" s="4"/>
+      <c r="G430" s="5"/>
       <c r="H430" s="4"/>
       <c r="I430" s="4"/>
     </row>
@@ -5250,7 +5250,7 @@
       <c r="D432" s="5"/>
       <c r="E432" s="4"/>
       <c r="F432" s="4"/>
-      <c r="G432" s="5"/>
+      <c r="G432" s="4"/>
       <c r="H432" s="4"/>
       <c r="I432" s="4"/>
     </row>
@@ -5261,7 +5261,7 @@
       <c r="D433" s="5"/>
       <c r="E433" s="4"/>
       <c r="F433" s="4"/>
-      <c r="G433" s="4"/>
+      <c r="G433" s="5"/>
       <c r="H433" s="4"/>
       <c r="I433" s="4"/>
     </row>
@@ -5327,7 +5327,7 @@
       <c r="D439" s="5"/>
       <c r="E439" s="4"/>
       <c r="F439" s="4"/>
-      <c r="G439" s="5"/>
+      <c r="G439" s="4"/>
       <c r="H439" s="4"/>
       <c r="I439" s="4"/>
     </row>
@@ -5338,7 +5338,7 @@
       <c r="D440" s="5"/>
       <c r="E440" s="4"/>
       <c r="F440" s="4"/>
-      <c r="G440" s="4"/>
+      <c r="G440" s="5"/>
       <c r="H440" s="4"/>
       <c r="I440" s="4"/>
     </row>
@@ -5382,7 +5382,7 @@
       <c r="D444" s="5"/>
       <c r="E444" s="4"/>
       <c r="F444" s="4"/>
-      <c r="G444" s="5"/>
+      <c r="G444" s="4"/>
       <c r="H444" s="4"/>
       <c r="I444" s="4"/>
     </row>
@@ -5393,7 +5393,7 @@
       <c r="D445" s="5"/>
       <c r="E445" s="4"/>
       <c r="F445" s="4"/>
-      <c r="G445" s="4"/>
+      <c r="G445" s="5"/>
       <c r="H445" s="4"/>
       <c r="I445" s="4"/>
     </row>
@@ -5404,7 +5404,7 @@
       <c r="D446" s="5"/>
       <c r="E446" s="4"/>
       <c r="F446" s="4"/>
-      <c r="G446" s="5"/>
+      <c r="G446" s="4"/>
       <c r="H446" s="4"/>
       <c r="I446" s="4"/>
     </row>
@@ -5415,7 +5415,7 @@
       <c r="D447" s="5"/>
       <c r="E447" s="4"/>
       <c r="F447" s="4"/>
-      <c r="G447" s="4"/>
+      <c r="G447" s="5"/>
       <c r="H447" s="4"/>
       <c r="I447" s="4"/>
     </row>
@@ -5426,7 +5426,7 @@
       <c r="D448" s="5"/>
       <c r="E448" s="4"/>
       <c r="F448" s="4"/>
-      <c r="G448" s="5"/>
+      <c r="G448" s="4"/>
       <c r="H448" s="4"/>
       <c r="I448" s="4"/>
     </row>
@@ -5437,7 +5437,7 @@
       <c r="D449" s="5"/>
       <c r="E449" s="4"/>
       <c r="F449" s="4"/>
-      <c r="G449" s="4"/>
+      <c r="G449" s="5"/>
       <c r="H449" s="4"/>
       <c r="I449" s="4"/>
     </row>
@@ -5558,7 +5558,7 @@
       <c r="D460" s="5"/>
       <c r="E460" s="4"/>
       <c r="F460" s="4"/>
-      <c r="G460" s="5"/>
+      <c r="G460" s="4"/>
       <c r="H460" s="4"/>
       <c r="I460" s="4"/>
     </row>
@@ -5569,7 +5569,7 @@
       <c r="D461" s="5"/>
       <c r="E461" s="4"/>
       <c r="F461" s="4"/>
-      <c r="G461" s="4"/>
+      <c r="G461" s="5"/>
       <c r="H461" s="4"/>
       <c r="I461" s="4"/>
     </row>
@@ -5602,7 +5602,7 @@
       <c r="D464" s="5"/>
       <c r="E464" s="4"/>
       <c r="F464" s="4"/>
-      <c r="G464" s="5"/>
+      <c r="G464" s="4"/>
       <c r="H464" s="4"/>
       <c r="I464" s="4"/>
     </row>
@@ -5613,7 +5613,7 @@
       <c r="D465" s="5"/>
       <c r="E465" s="4"/>
       <c r="F465" s="4"/>
-      <c r="G465" s="4"/>
+      <c r="G465" s="5"/>
       <c r="H465" s="4"/>
       <c r="I465" s="4"/>
     </row>
@@ -5756,7 +5756,7 @@
       <c r="D478" s="5"/>
       <c r="E478" s="4"/>
       <c r="F478" s="4"/>
-      <c r="G478" s="5"/>
+      <c r="G478" s="4"/>
       <c r="H478" s="4"/>
       <c r="I478" s="4"/>
     </row>
@@ -5767,7 +5767,7 @@
       <c r="D479" s="5"/>
       <c r="E479" s="4"/>
       <c r="F479" s="4"/>
-      <c r="G479" s="4"/>
+      <c r="G479" s="5"/>
       <c r="H479" s="4"/>
       <c r="I479" s="4"/>
     </row>
@@ -5899,7 +5899,7 @@
       <c r="D491" s="5"/>
       <c r="E491" s="4"/>
       <c r="F491" s="4"/>
-      <c r="G491" s="5"/>
+      <c r="G491" s="4"/>
       <c r="H491" s="4"/>
       <c r="I491" s="4"/>
     </row>
@@ -5910,7 +5910,7 @@
       <c r="D492" s="5"/>
       <c r="E492" s="4"/>
       <c r="F492" s="4"/>
-      <c r="G492" s="4"/>
+      <c r="G492" s="5"/>
       <c r="H492" s="4"/>
       <c r="I492" s="4"/>
     </row>
@@ -5987,7 +5987,7 @@
       <c r="D499" s="5"/>
       <c r="E499" s="4"/>
       <c r="F499" s="4"/>
-      <c r="G499" s="5"/>
+      <c r="G499" s="4"/>
       <c r="H499" s="4"/>
       <c r="I499" s="4"/>
     </row>
@@ -5998,7 +5998,7 @@
       <c r="D500" s="5"/>
       <c r="E500" s="4"/>
       <c r="F500" s="4"/>
-      <c r="G500" s="4"/>
+      <c r="G500" s="5"/>
       <c r="H500" s="4"/>
       <c r="I500" s="4"/>
     </row>
@@ -6009,7 +6009,7 @@
       <c r="D501" s="5"/>
       <c r="E501" s="4"/>
       <c r="F501" s="4"/>
-      <c r="G501" s="5"/>
+      <c r="G501" s="4"/>
       <c r="H501" s="4"/>
       <c r="I501" s="4"/>
     </row>
@@ -6020,7 +6020,7 @@
       <c r="D502" s="5"/>
       <c r="E502" s="4"/>
       <c r="F502" s="4"/>
-      <c r="G502" s="4"/>
+      <c r="G502" s="5"/>
       <c r="H502" s="4"/>
       <c r="I502" s="4"/>
     </row>
@@ -6053,7 +6053,7 @@
       <c r="D505" s="5"/>
       <c r="E505" s="4"/>
       <c r="F505" s="4"/>
-      <c r="G505" s="5"/>
+      <c r="G505" s="4"/>
       <c r="H505" s="4"/>
       <c r="I505" s="4"/>
     </row>
@@ -6064,7 +6064,7 @@
       <c r="D506" s="5"/>
       <c r="E506" s="4"/>
       <c r="F506" s="4"/>
-      <c r="G506" s="4"/>
+      <c r="G506" s="5"/>
       <c r="H506" s="4"/>
       <c r="I506" s="4"/>
     </row>
@@ -6394,7 +6394,7 @@
       <c r="D536" s="5"/>
       <c r="E536" s="4"/>
       <c r="F536" s="4"/>
-      <c r="G536" s="5"/>
+      <c r="G536" s="4"/>
       <c r="H536" s="4"/>
       <c r="I536" s="4"/>
     </row>
@@ -6405,7 +6405,7 @@
       <c r="D537" s="5"/>
       <c r="E537" s="4"/>
       <c r="F537" s="4"/>
-      <c r="G537" s="4"/>
+      <c r="G537" s="5"/>
       <c r="H537" s="4"/>
       <c r="I537" s="4"/>
     </row>
@@ -6504,7 +6504,7 @@
       <c r="D546" s="5"/>
       <c r="E546" s="4"/>
       <c r="F546" s="4"/>
-      <c r="G546" s="5"/>
+      <c r="G546" s="4"/>
       <c r="H546" s="4"/>
       <c r="I546" s="4"/>
     </row>
@@ -6515,7 +6515,7 @@
       <c r="D547" s="5"/>
       <c r="E547" s="4"/>
       <c r="F547" s="4"/>
-      <c r="G547" s="4"/>
+      <c r="G547" s="5"/>
       <c r="H547" s="4"/>
       <c r="I547" s="4"/>
     </row>
@@ -6570,7 +6570,7 @@
       <c r="D552" s="5"/>
       <c r="E552" s="4"/>
       <c r="F552" s="4"/>
-      <c r="G552" s="5"/>
+      <c r="G552" s="4"/>
       <c r="H552" s="4"/>
       <c r="I552" s="4"/>
     </row>
@@ -6581,7 +6581,7 @@
       <c r="D553" s="5"/>
       <c r="E553" s="4"/>
       <c r="F553" s="4"/>
-      <c r="G553" s="4"/>
+      <c r="G553" s="5"/>
       <c r="H553" s="4"/>
       <c r="I553" s="4"/>
     </row>
@@ -6680,7 +6680,7 @@
       <c r="D562" s="5"/>
       <c r="E562" s="4"/>
       <c r="F562" s="4"/>
-      <c r="G562" s="5"/>
+      <c r="G562" s="4"/>
       <c r="H562" s="4"/>
       <c r="I562" s="4"/>
     </row>
@@ -6691,7 +6691,7 @@
       <c r="D563" s="5"/>
       <c r="E563" s="4"/>
       <c r="F563" s="4"/>
-      <c r="G563" s="4"/>
+      <c r="G563" s="5"/>
       <c r="H563" s="4"/>
       <c r="I563" s="4"/>
     </row>
@@ -6735,7 +6735,7 @@
       <c r="D567" s="5"/>
       <c r="E567" s="4"/>
       <c r="F567" s="4"/>
-      <c r="G567" s="5"/>
+      <c r="G567" s="4"/>
       <c r="H567" s="4"/>
       <c r="I567" s="4"/>
     </row>
@@ -6746,7 +6746,7 @@
       <c r="D568" s="5"/>
       <c r="E568" s="4"/>
       <c r="F568" s="4"/>
-      <c r="G568" s="4"/>
+      <c r="G568" s="5"/>
       <c r="H568" s="4"/>
       <c r="I568" s="4"/>
     </row>
@@ -6790,7 +6790,7 @@
       <c r="D572" s="5"/>
       <c r="E572" s="4"/>
       <c r="F572" s="4"/>
-      <c r="G572" s="5"/>
+      <c r="G572" s="4"/>
       <c r="H572" s="4"/>
       <c r="I572" s="4"/>
     </row>
@@ -6801,7 +6801,7 @@
       <c r="D573" s="5"/>
       <c r="E573" s="4"/>
       <c r="F573" s="4"/>
-      <c r="G573" s="4"/>
+      <c r="G573" s="5"/>
       <c r="H573" s="4"/>
       <c r="I573" s="4"/>
     </row>
@@ -6834,7 +6834,7 @@
       <c r="D576" s="5"/>
       <c r="E576" s="4"/>
       <c r="F576" s="4"/>
-      <c r="G576" s="5"/>
+      <c r="G576" s="4"/>
       <c r="H576" s="4"/>
       <c r="I576" s="4"/>
     </row>
@@ -6856,7 +6856,7 @@
       <c r="D578" s="5"/>
       <c r="E578" s="4"/>
       <c r="F578" s="4"/>
-      <c r="G578" s="4"/>
+      <c r="G578" s="5"/>
       <c r="H578" s="4"/>
       <c r="I578" s="4"/>
     </row>
@@ -6889,7 +6889,7 @@
       <c r="D581" s="5"/>
       <c r="E581" s="4"/>
       <c r="F581" s="4"/>
-      <c r="G581" s="5"/>
+      <c r="G581" s="4"/>
       <c r="H581" s="4"/>
       <c r="I581" s="4"/>
     </row>
@@ -6900,7 +6900,7 @@
       <c r="D582" s="5"/>
       <c r="E582" s="4"/>
       <c r="F582" s="4"/>
-      <c r="G582" s="4"/>
+      <c r="G582" s="5"/>
       <c r="H582" s="4"/>
       <c r="I582" s="4"/>
     </row>
@@ -6911,7 +6911,7 @@
       <c r="D583" s="5"/>
       <c r="E583" s="4"/>
       <c r="F583" s="4"/>
-      <c r="G583" s="5"/>
+      <c r="G583" s="4"/>
       <c r="H583" s="4"/>
       <c r="I583" s="4"/>
     </row>
@@ -6922,7 +6922,7 @@
       <c r="D584" s="5"/>
       <c r="E584" s="4"/>
       <c r="F584" s="4"/>
-      <c r="G584" s="4"/>
+      <c r="G584" s="5"/>
       <c r="H584" s="4"/>
       <c r="I584" s="4"/>
     </row>
@@ -7010,7 +7010,7 @@
       <c r="D592" s="5"/>
       <c r="E592" s="4"/>
       <c r="F592" s="4"/>
-      <c r="G592" s="5"/>
+      <c r="G592" s="4"/>
       <c r="H592" s="4"/>
       <c r="I592" s="4"/>
     </row>
@@ -7021,7 +7021,7 @@
       <c r="D593" s="5"/>
       <c r="E593" s="4"/>
       <c r="F593" s="4"/>
-      <c r="G593" s="4"/>
+      <c r="G593" s="5"/>
       <c r="H593" s="4"/>
       <c r="I593" s="4"/>
     </row>
@@ -7065,7 +7065,7 @@
       <c r="D597" s="5"/>
       <c r="E597" s="4"/>
       <c r="F597" s="4"/>
-      <c r="G597" s="5"/>
+      <c r="G597" s="4"/>
       <c r="H597" s="4"/>
       <c r="I597" s="4"/>
     </row>
@@ -7076,7 +7076,7 @@
       <c r="D598" s="5"/>
       <c r="E598" s="4"/>
       <c r="F598" s="4"/>
-      <c r="G598" s="4"/>
+      <c r="G598" s="5"/>
       <c r="H598" s="4"/>
       <c r="I598" s="4"/>
     </row>
@@ -7142,7 +7142,7 @@
       <c r="D604" s="5"/>
       <c r="E604" s="4"/>
       <c r="F604" s="4"/>
-      <c r="G604" s="5"/>
+      <c r="G604" s="4"/>
       <c r="H604" s="4"/>
       <c r="I604" s="4"/>
     </row>
@@ -7153,7 +7153,7 @@
       <c r="D605" s="5"/>
       <c r="E605" s="4"/>
       <c r="F605" s="4"/>
-      <c r="G605" s="4"/>
+      <c r="G605" s="5"/>
       <c r="H605" s="4"/>
       <c r="I605" s="4"/>
     </row>
@@ -7186,7 +7186,7 @@
       <c r="D608" s="5"/>
       <c r="E608" s="4"/>
       <c r="F608" s="4"/>
-      <c r="G608" s="5"/>
+      <c r="G608" s="4"/>
       <c r="H608" s="4"/>
       <c r="I608" s="4"/>
     </row>
@@ -7197,7 +7197,7 @@
       <c r="D609" s="5"/>
       <c r="E609" s="4"/>
       <c r="F609" s="4"/>
-      <c r="G609" s="4"/>
+      <c r="G609" s="5"/>
       <c r="H609" s="4"/>
       <c r="I609" s="4"/>
     </row>
@@ -7230,7 +7230,7 @@
       <c r="D612" s="5"/>
       <c r="E612" s="4"/>
       <c r="F612" s="4"/>
-      <c r="G612" s="5"/>
+      <c r="G612" s="4"/>
       <c r="H612" s="4"/>
       <c r="I612" s="4"/>
     </row>
@@ -7241,7 +7241,7 @@
       <c r="D613" s="5"/>
       <c r="E613" s="4"/>
       <c r="F613" s="4"/>
-      <c r="G613" s="4"/>
+      <c r="G613" s="5"/>
       <c r="H613" s="4"/>
       <c r="I613" s="4"/>
     </row>
@@ -7252,7 +7252,7 @@
       <c r="D614" s="5"/>
       <c r="E614" s="4"/>
       <c r="F614" s="4"/>
-      <c r="G614" s="5"/>
+      <c r="G614" s="4"/>
       <c r="H614" s="4"/>
       <c r="I614" s="4"/>
     </row>
@@ -7263,7 +7263,7 @@
       <c r="D615" s="5"/>
       <c r="E615" s="4"/>
       <c r="F615" s="4"/>
-      <c r="G615" s="4"/>
+      <c r="G615" s="5"/>
       <c r="H615" s="4"/>
       <c r="I615" s="4"/>
     </row>
@@ -7307,7 +7307,7 @@
       <c r="D619" s="5"/>
       <c r="E619" s="4"/>
       <c r="F619" s="4"/>
-      <c r="G619" s="5"/>
+      <c r="G619" s="4"/>
       <c r="H619" s="4"/>
       <c r="I619" s="4"/>
     </row>
@@ -7329,7 +7329,7 @@
       <c r="D621" s="5"/>
       <c r="E621" s="4"/>
       <c r="F621" s="4"/>
-      <c r="G621" s="4"/>
+      <c r="G621" s="5"/>
       <c r="H621" s="4"/>
       <c r="I621" s="4"/>
     </row>
@@ -7351,7 +7351,7 @@
       <c r="D623" s="5"/>
       <c r="E623" s="4"/>
       <c r="F623" s="4"/>
-      <c r="G623" s="5"/>
+      <c r="G623" s="4"/>
       <c r="H623" s="4"/>
       <c r="I623" s="4"/>
     </row>
@@ -7362,7 +7362,7 @@
       <c r="D624" s="5"/>
       <c r="E624" s="4"/>
       <c r="F624" s="4"/>
-      <c r="G624" s="4"/>
+      <c r="G624" s="5"/>
       <c r="H624" s="4"/>
       <c r="I624" s="4"/>
     </row>
@@ -7439,7 +7439,7 @@
       <c r="D631" s="5"/>
       <c r="E631" s="4"/>
       <c r="F631" s="4"/>
-      <c r="G631" s="5"/>
+      <c r="G631" s="4"/>
       <c r="H631" s="4"/>
       <c r="I631" s="4"/>
     </row>
@@ -7450,7 +7450,7 @@
       <c r="D632" s="5"/>
       <c r="E632" s="4"/>
       <c r="F632" s="4"/>
-      <c r="G632" s="4"/>
+      <c r="G632" s="5"/>
       <c r="H632" s="4"/>
       <c r="I632" s="4"/>
     </row>
@@ -7472,7 +7472,7 @@
       <c r="D634" s="5"/>
       <c r="E634" s="4"/>
       <c r="F634" s="4"/>
-      <c r="G634" s="5"/>
+      <c r="G634" s="4"/>
       <c r="H634" s="4"/>
       <c r="I634" s="4"/>
     </row>
@@ -7483,7 +7483,7 @@
       <c r="D635" s="5"/>
       <c r="E635" s="4"/>
       <c r="F635" s="4"/>
-      <c r="G635" s="4"/>
+      <c r="G635" s="5"/>
       <c r="H635" s="4"/>
       <c r="I635" s="4"/>
     </row>
@@ -7527,7 +7527,7 @@
       <c r="D639" s="5"/>
       <c r="E639" s="4"/>
       <c r="F639" s="4"/>
-      <c r="G639" s="5"/>
+      <c r="G639" s="4"/>
       <c r="H639" s="4"/>
       <c r="I639" s="4"/>
     </row>
@@ -7538,7 +7538,7 @@
       <c r="D640" s="5"/>
       <c r="E640" s="4"/>
       <c r="F640" s="4"/>
-      <c r="G640" s="4"/>
+      <c r="G640" s="5"/>
       <c r="H640" s="4"/>
       <c r="I640" s="4"/>
     </row>
@@ -7648,7 +7648,7 @@
       <c r="D650" s="5"/>
       <c r="E650" s="4"/>
       <c r="F650" s="4"/>
-      <c r="G650" s="5"/>
+      <c r="G650" s="4"/>
       <c r="H650" s="4"/>
       <c r="I650" s="4"/>
     </row>
@@ -7659,7 +7659,7 @@
       <c r="D651" s="5"/>
       <c r="E651" s="4"/>
       <c r="F651" s="4"/>
-      <c r="G651" s="4"/>
+      <c r="G651" s="5"/>
       <c r="H651" s="4"/>
       <c r="I651" s="4"/>
     </row>
@@ -7692,7 +7692,7 @@
       <c r="D654" s="5"/>
       <c r="E654" s="4"/>
       <c r="F654" s="4"/>
-      <c r="G654" s="5"/>
+      <c r="G654" s="4"/>
       <c r="H654" s="4"/>
       <c r="I654" s="4"/>
     </row>
@@ -7703,7 +7703,7 @@
       <c r="D655" s="5"/>
       <c r="E655" s="4"/>
       <c r="F655" s="4"/>
-      <c r="G655" s="4"/>
+      <c r="G655" s="5"/>
       <c r="H655" s="4"/>
       <c r="I655" s="4"/>
     </row>
@@ -7747,7 +7747,7 @@
       <c r="D659" s="5"/>
       <c r="E659" s="4"/>
       <c r="F659" s="4"/>
-      <c r="G659" s="5"/>
+      <c r="G659" s="4"/>
       <c r="H659" s="4"/>
       <c r="I659" s="4"/>
     </row>
@@ -7758,7 +7758,7 @@
       <c r="D660" s="5"/>
       <c r="E660" s="4"/>
       <c r="F660" s="4"/>
-      <c r="G660" s="4"/>
+      <c r="G660" s="5"/>
       <c r="H660" s="4"/>
       <c r="I660" s="4"/>
     </row>
@@ -7901,7 +7901,7 @@
       <c r="D673" s="5"/>
       <c r="E673" s="4"/>
       <c r="F673" s="4"/>
-      <c r="G673" s="5"/>
+      <c r="G673" s="4"/>
       <c r="H673" s="4"/>
       <c r="I673" s="4"/>
     </row>
@@ -7923,7 +7923,7 @@
       <c r="D675" s="5"/>
       <c r="E675" s="4"/>
       <c r="F675" s="4"/>
-      <c r="G675" s="4"/>
+      <c r="G675" s="5"/>
       <c r="H675" s="4"/>
       <c r="I675" s="4"/>
     </row>
@@ -8022,7 +8022,7 @@
       <c r="D684" s="5"/>
       <c r="E684" s="4"/>
       <c r="F684" s="4"/>
-      <c r="G684" s="5"/>
+      <c r="G684" s="4"/>
       <c r="H684" s="4"/>
       <c r="I684" s="4"/>
     </row>
@@ -8033,7 +8033,7 @@
       <c r="D685" s="5"/>
       <c r="E685" s="4"/>
       <c r="F685" s="4"/>
-      <c r="G685" s="4"/>
+      <c r="G685" s="5"/>
       <c r="H685" s="4"/>
       <c r="I685" s="4"/>
     </row>
@@ -8088,7 +8088,7 @@
       <c r="D690" s="5"/>
       <c r="E690" s="4"/>
       <c r="F690" s="4"/>
-      <c r="G690" s="5"/>
+      <c r="G690" s="4"/>
       <c r="H690" s="4"/>
       <c r="I690" s="4"/>
     </row>
@@ -8099,7 +8099,7 @@
       <c r="D691" s="5"/>
       <c r="E691" s="4"/>
       <c r="F691" s="4"/>
-      <c r="G691" s="4"/>
+      <c r="G691" s="5"/>
       <c r="H691" s="4"/>
       <c r="I691" s="4"/>
     </row>
@@ -8198,7 +8198,7 @@
       <c r="D700" s="5"/>
       <c r="E700" s="4"/>
       <c r="F700" s="4"/>
-      <c r="G700" s="5"/>
+      <c r="G700" s="4"/>
       <c r="H700" s="4"/>
       <c r="I700" s="4"/>
     </row>
@@ -8209,7 +8209,7 @@
       <c r="D701" s="5"/>
       <c r="E701" s="4"/>
       <c r="F701" s="4"/>
-      <c r="G701" s="4"/>
+      <c r="G701" s="5"/>
       <c r="H701" s="4"/>
       <c r="I701" s="4"/>
     </row>
@@ -8319,7 +8319,7 @@
       <c r="D711" s="5"/>
       <c r="E711" s="4"/>
       <c r="F711" s="4"/>
-      <c r="G711" s="5"/>
+      <c r="G711" s="4"/>
       <c r="H711" s="4"/>
       <c r="I711" s="4"/>
     </row>
@@ -8330,7 +8330,7 @@
       <c r="D712" s="5"/>
       <c r="E712" s="4"/>
       <c r="F712" s="4"/>
-      <c r="G712" s="4"/>
+      <c r="G712" s="5"/>
       <c r="H712" s="4"/>
       <c r="I712" s="4"/>
     </row>
@@ -8363,7 +8363,7 @@
       <c r="D715" s="5"/>
       <c r="E715" s="4"/>
       <c r="F715" s="4"/>
-      <c r="G715" s="5"/>
+      <c r="G715" s="4"/>
       <c r="H715" s="4"/>
       <c r="I715" s="4"/>
     </row>
@@ -8374,7 +8374,7 @@
       <c r="D716" s="5"/>
       <c r="E716" s="4"/>
       <c r="F716" s="4"/>
-      <c r="G716" s="4"/>
+      <c r="G716" s="5"/>
       <c r="H716" s="4"/>
       <c r="I716" s="4"/>
     </row>
@@ -8407,7 +8407,7 @@
       <c r="D719" s="5"/>
       <c r="E719" s="4"/>
       <c r="F719" s="4"/>
-      <c r="G719" s="5"/>
+      <c r="G719" s="4"/>
       <c r="H719" s="4"/>
       <c r="I719" s="4"/>
     </row>
@@ -8429,7 +8429,7 @@
       <c r="D721" s="5"/>
       <c r="E721" s="4"/>
       <c r="F721" s="4"/>
-      <c r="G721" s="4"/>
+      <c r="G721" s="5"/>
       <c r="H721" s="4"/>
       <c r="I721" s="4"/>
     </row>
@@ -8440,7 +8440,7 @@
       <c r="D722" s="5"/>
       <c r="E722" s="4"/>
       <c r="F722" s="4"/>
-      <c r="G722" s="5"/>
+      <c r="G722" s="4"/>
       <c r="H722" s="4"/>
       <c r="I722" s="4"/>
     </row>
@@ -8451,7 +8451,7 @@
       <c r="D723" s="5"/>
       <c r="E723" s="4"/>
       <c r="F723" s="4"/>
-      <c r="G723" s="4"/>
+      <c r="G723" s="5"/>
       <c r="H723" s="4"/>
       <c r="I723" s="4"/>
     </row>
@@ -8462,7 +8462,7 @@
       <c r="D724" s="5"/>
       <c r="E724" s="4"/>
       <c r="F724" s="4"/>
-      <c r="G724" s="5"/>
+      <c r="G724" s="4"/>
       <c r="H724" s="4"/>
       <c r="I724" s="4"/>
     </row>
@@ -8473,7 +8473,7 @@
       <c r="D725" s="5"/>
       <c r="E725" s="4"/>
       <c r="F725" s="4"/>
-      <c r="G725" s="4"/>
+      <c r="G725" s="5"/>
       <c r="H725" s="4"/>
       <c r="I725" s="4"/>
     </row>
@@ -8572,7 +8572,7 @@
       <c r="D734" s="5"/>
       <c r="E734" s="4"/>
       <c r="F734" s="4"/>
-      <c r="G734" s="5"/>
+      <c r="G734" s="4"/>
       <c r="H734" s="4"/>
       <c r="I734" s="4"/>
     </row>
@@ -8583,7 +8583,7 @@
       <c r="D735" s="5"/>
       <c r="E735" s="4"/>
       <c r="F735" s="4"/>
-      <c r="G735" s="4"/>
+      <c r="G735" s="5"/>
       <c r="H735" s="4"/>
       <c r="I735" s="4"/>
     </row>
@@ -8594,7 +8594,7 @@
       <c r="D736" s="5"/>
       <c r="E736" s="4"/>
       <c r="F736" s="4"/>
-      <c r="G736" s="5"/>
+      <c r="G736" s="4"/>
       <c r="H736" s="4"/>
       <c r="I736" s="4"/>
     </row>
@@ -8605,7 +8605,7 @@
       <c r="D737" s="5"/>
       <c r="E737" s="4"/>
       <c r="F737" s="4"/>
-      <c r="G737" s="4"/>
+      <c r="G737" s="5"/>
       <c r="H737" s="4"/>
       <c r="I737" s="4"/>
     </row>
@@ -8693,7 +8693,7 @@
       <c r="D745" s="5"/>
       <c r="E745" s="4"/>
       <c r="F745" s="4"/>
-      <c r="G745" s="5"/>
+      <c r="G745" s="4"/>
       <c r="H745" s="4"/>
       <c r="I745" s="4"/>
     </row>
@@ -8704,7 +8704,7 @@
       <c r="D746" s="5"/>
       <c r="E746" s="4"/>
       <c r="F746" s="4"/>
-      <c r="G746" s="4"/>
+      <c r="G746" s="5"/>
       <c r="H746" s="4"/>
       <c r="I746" s="4"/>
     </row>
@@ -8737,7 +8737,7 @@
       <c r="D749" s="5"/>
       <c r="E749" s="4"/>
       <c r="F749" s="4"/>
-      <c r="G749" s="5"/>
+      <c r="G749" s="4"/>
       <c r="H749" s="4"/>
       <c r="I749" s="4"/>
     </row>
@@ -8748,7 +8748,7 @@
       <c r="D750" s="5"/>
       <c r="E750" s="4"/>
       <c r="F750" s="4"/>
-      <c r="G750" s="4"/>
+      <c r="G750" s="5"/>
       <c r="H750" s="4"/>
       <c r="I750" s="4"/>
     </row>
@@ -8979,7 +8979,7 @@
       <c r="D771" s="5"/>
       <c r="E771" s="4"/>
       <c r="F771" s="4"/>
-      <c r="G771" s="5"/>
+      <c r="G771" s="4"/>
       <c r="H771" s="4"/>
       <c r="I771" s="4"/>
     </row>
@@ -8990,7 +8990,7 @@
       <c r="D772" s="5"/>
       <c r="E772" s="4"/>
       <c r="F772" s="4"/>
-      <c r="G772" s="4"/>
+      <c r="G772" s="5"/>
       <c r="H772" s="4"/>
       <c r="I772" s="4"/>
     </row>
@@ -9001,7 +9001,7 @@
       <c r="D773" s="5"/>
       <c r="E773" s="4"/>
       <c r="F773" s="4"/>
-      <c r="G773" s="5"/>
+      <c r="G773" s="4"/>
       <c r="H773" s="4"/>
       <c r="I773" s="4"/>
     </row>
@@ -9012,7 +9012,7 @@
       <c r="D774" s="5"/>
       <c r="E774" s="4"/>
       <c r="F774" s="4"/>
-      <c r="G774" s="4"/>
+      <c r="G774" s="5"/>
       <c r="H774" s="4"/>
       <c r="I774" s="4"/>
     </row>
@@ -9045,7 +9045,7 @@
       <c r="D777" s="5"/>
       <c r="E777" s="4"/>
       <c r="F777" s="4"/>
-      <c r="G777" s="5"/>
+      <c r="G777" s="4"/>
       <c r="H777" s="4"/>
       <c r="I777" s="4"/>
     </row>
@@ -9056,7 +9056,7 @@
       <c r="D778" s="5"/>
       <c r="E778" s="4"/>
       <c r="F778" s="4"/>
-      <c r="G778" s="4"/>
+      <c r="G778" s="5"/>
       <c r="H778" s="4"/>
       <c r="I778" s="4"/>
     </row>
@@ -9100,7 +9100,7 @@
       <c r="D782" s="5"/>
       <c r="E782" s="4"/>
       <c r="F782" s="4"/>
-      <c r="G782" s="5"/>
+      <c r="G782" s="4"/>
       <c r="H782" s="4"/>
       <c r="I782" s="4"/>
     </row>
@@ -9111,7 +9111,7 @@
       <c r="D783" s="5"/>
       <c r="E783" s="4"/>
       <c r="F783" s="4"/>
-      <c r="G783" s="4"/>
+      <c r="G783" s="5"/>
       <c r="H783" s="4"/>
       <c r="I783" s="4"/>
     </row>
@@ -9177,7 +9177,7 @@
       <c r="D789" s="5"/>
       <c r="E789" s="4"/>
       <c r="F789" s="4"/>
-      <c r="G789" s="5"/>
+      <c r="G789" s="4"/>
       <c r="H789" s="4"/>
       <c r="I789" s="4"/>
     </row>
@@ -9188,7 +9188,7 @@
       <c r="D790" s="5"/>
       <c r="E790" s="4"/>
       <c r="F790" s="4"/>
-      <c r="G790" s="4"/>
+      <c r="G790" s="5"/>
       <c r="H790" s="4"/>
       <c r="I790" s="4"/>
     </row>
@@ -9298,7 +9298,7 @@
       <c r="D800" s="5"/>
       <c r="E800" s="4"/>
       <c r="F800" s="4"/>
-      <c r="G800" s="5"/>
+      <c r="G800" s="4"/>
       <c r="H800" s="4"/>
       <c r="I800" s="4"/>
     </row>
@@ -9309,7 +9309,7 @@
       <c r="D801" s="5"/>
       <c r="E801" s="4"/>
       <c r="F801" s="4"/>
-      <c r="G801" s="4"/>
+      <c r="G801" s="5"/>
       <c r="H801" s="4"/>
       <c r="I801" s="4"/>
     </row>
@@ -9331,7 +9331,7 @@
       <c r="D803" s="5"/>
       <c r="E803" s="4"/>
       <c r="F803" s="4"/>
-      <c r="G803" s="5"/>
+      <c r="G803" s="4"/>
       <c r="H803" s="4"/>
       <c r="I803" s="4"/>
     </row>
@@ -9342,7 +9342,7 @@
       <c r="D804" s="5"/>
       <c r="E804" s="4"/>
       <c r="F804" s="4"/>
-      <c r="G804" s="4"/>
+      <c r="G804" s="5"/>
       <c r="H804" s="4"/>
       <c r="I804" s="4"/>
     </row>
@@ -9353,7 +9353,7 @@
       <c r="D805" s="5"/>
       <c r="E805" s="4"/>
       <c r="F805" s="4"/>
-      <c r="G805" s="5"/>
+      <c r="G805" s="4"/>
       <c r="H805" s="4"/>
       <c r="I805" s="4"/>
     </row>
@@ -9364,7 +9364,7 @@
       <c r="D806" s="5"/>
       <c r="E806" s="4"/>
       <c r="F806" s="4"/>
-      <c r="G806" s="4"/>
+      <c r="G806" s="5"/>
       <c r="H806" s="4"/>
       <c r="I806" s="4"/>
     </row>
@@ -9408,7 +9408,7 @@
       <c r="D810" s="5"/>
       <c r="E810" s="4"/>
       <c r="F810" s="4"/>
-      <c r="G810" s="5"/>
+      <c r="G810" s="4"/>
       <c r="H810" s="4"/>
       <c r="I810" s="4"/>
     </row>
@@ -9419,7 +9419,7 @@
       <c r="D811" s="5"/>
       <c r="E811" s="4"/>
       <c r="F811" s="4"/>
-      <c r="G811" s="4"/>
+      <c r="G811" s="5"/>
       <c r="H811" s="4"/>
       <c r="I811" s="4"/>
     </row>
@@ -9430,7 +9430,7 @@
       <c r="D812" s="5"/>
       <c r="E812" s="4"/>
       <c r="F812" s="4"/>
-      <c r="G812" s="5"/>
+      <c r="G812" s="4"/>
       <c r="H812" s="4"/>
       <c r="I812" s="4"/>
     </row>
@@ -9452,7 +9452,7 @@
       <c r="D814" s="5"/>
       <c r="E814" s="4"/>
       <c r="F814" s="4"/>
-      <c r="G814" s="4"/>
+      <c r="G814" s="5"/>
       <c r="H814" s="4"/>
       <c r="I814" s="4"/>
     </row>
@@ -9507,7 +9507,7 @@
       <c r="D819" s="5"/>
       <c r="E819" s="4"/>
       <c r="F819" s="4"/>
-      <c r="G819" s="5"/>
+      <c r="G819" s="4"/>
       <c r="H819" s="4"/>
       <c r="I819" s="4"/>
     </row>
@@ -9518,7 +9518,7 @@
       <c r="D820" s="5"/>
       <c r="E820" s="4"/>
       <c r="F820" s="4"/>
-      <c r="G820" s="4"/>
+      <c r="G820" s="5"/>
       <c r="H820" s="4"/>
       <c r="I820" s="4"/>
     </row>
@@ -9584,7 +9584,7 @@
       <c r="D826" s="5"/>
       <c r="E826" s="4"/>
       <c r="F826" s="4"/>
-      <c r="G826" s="5"/>
+      <c r="G826" s="4"/>
       <c r="H826" s="4"/>
       <c r="I826" s="4"/>
     </row>
@@ -9595,7 +9595,7 @@
       <c r="D827" s="5"/>
       <c r="E827" s="4"/>
       <c r="F827" s="4"/>
-      <c r="G827" s="4"/>
+      <c r="G827" s="5"/>
       <c r="H827" s="4"/>
       <c r="I827" s="4"/>
     </row>
@@ -9650,7 +9650,7 @@
       <c r="D832" s="5"/>
       <c r="E832" s="4"/>
       <c r="F832" s="4"/>
-      <c r="G832" s="5"/>
+      <c r="G832" s="4"/>
       <c r="H832" s="4"/>
       <c r="I832" s="4"/>
     </row>
@@ -9661,7 +9661,7 @@
       <c r="D833" s="5"/>
       <c r="E833" s="4"/>
       <c r="F833" s="4"/>
-      <c r="G833" s="4"/>
+      <c r="G833" s="5"/>
       <c r="H833" s="4"/>
       <c r="I833" s="4"/>
     </row>
@@ -9683,7 +9683,7 @@
       <c r="D835" s="5"/>
       <c r="E835" s="4"/>
       <c r="F835" s="4"/>
-      <c r="G835" s="5"/>
+      <c r="G835" s="4"/>
       <c r="H835" s="4"/>
       <c r="I835" s="4"/>
     </row>
@@ -9705,7 +9705,7 @@
       <c r="D837" s="5"/>
       <c r="E837" s="4"/>
       <c r="F837" s="4"/>
-      <c r="G837" s="4"/>
+      <c r="G837" s="5"/>
       <c r="H837" s="4"/>
       <c r="I837" s="4"/>
     </row>
@@ -9727,7 +9727,7 @@
       <c r="D839" s="5"/>
       <c r="E839" s="4"/>
       <c r="F839" s="4"/>
-      <c r="G839" s="5"/>
+      <c r="G839" s="4"/>
       <c r="H839" s="4"/>
       <c r="I839" s="4"/>
     </row>
@@ -9760,7 +9760,7 @@
       <c r="D842" s="5"/>
       <c r="E842" s="4"/>
       <c r="F842" s="4"/>
-      <c r="G842" s="4"/>
+      <c r="G842" s="5"/>
       <c r="H842" s="4"/>
       <c r="I842" s="4"/>
     </row>
@@ -9815,7 +9815,7 @@
       <c r="D847" s="5"/>
       <c r="E847" s="4"/>
       <c r="F847" s="4"/>
-      <c r="G847" s="5"/>
+      <c r="G847" s="4"/>
       <c r="H847" s="4"/>
       <c r="I847" s="4"/>
     </row>
@@ -9826,7 +9826,7 @@
       <c r="D848" s="5"/>
       <c r="E848" s="4"/>
       <c r="F848" s="4"/>
-      <c r="G848" s="4"/>
+      <c r="G848" s="5"/>
       <c r="H848" s="4"/>
       <c r="I848" s="4"/>
     </row>
@@ -10035,7 +10035,7 @@
       <c r="D867" s="5"/>
       <c r="E867" s="4"/>
       <c r="F867" s="4"/>
-      <c r="G867" s="5"/>
+      <c r="G867" s="4"/>
       <c r="H867" s="4"/>
       <c r="I867" s="4"/>
     </row>
@@ -10046,7 +10046,7 @@
       <c r="D868" s="5"/>
       <c r="E868" s="4"/>
       <c r="F868" s="4"/>
-      <c r="G868" s="4"/>
+      <c r="G868" s="5"/>
       <c r="H868" s="4"/>
       <c r="I868" s="4"/>
     </row>
@@ -10222,7 +10222,7 @@
       <c r="D884" s="5"/>
       <c r="E884" s="4"/>
       <c r="F884" s="4"/>
-      <c r="G884" s="5"/>
+      <c r="G884" s="4"/>
       <c r="H884" s="4"/>
       <c r="I884" s="4"/>
     </row>
@@ -10244,7 +10244,7 @@
       <c r="D886" s="5"/>
       <c r="E886" s="4"/>
       <c r="F886" s="4"/>
-      <c r="G886" s="4"/>
+      <c r="G886" s="5"/>
       <c r="H886" s="4"/>
       <c r="I886" s="4"/>
     </row>
@@ -10277,7 +10277,7 @@
       <c r="D889" s="5"/>
       <c r="E889" s="4"/>
       <c r="F889" s="4"/>
-      <c r="G889" s="5"/>
+      <c r="G889" s="4"/>
       <c r="H889" s="4"/>
       <c r="I889" s="4"/>
     </row>
@@ -10288,7 +10288,7 @@
       <c r="D890" s="5"/>
       <c r="E890" s="4"/>
       <c r="F890" s="4"/>
-      <c r="G890" s="4"/>
+      <c r="G890" s="5"/>
       <c r="H890" s="4"/>
       <c r="I890" s="4"/>
     </row>
@@ -10332,7 +10332,7 @@
       <c r="D894" s="5"/>
       <c r="E894" s="4"/>
       <c r="F894" s="4"/>
-      <c r="G894" s="5"/>
+      <c r="G894" s="4"/>
       <c r="H894" s="4"/>
       <c r="I894" s="4"/>
     </row>
@@ -10343,7 +10343,7 @@
       <c r="D895" s="5"/>
       <c r="E895" s="4"/>
       <c r="F895" s="4"/>
-      <c r="G895" s="4"/>
+      <c r="G895" s="5"/>
       <c r="H895" s="4"/>
       <c r="I895" s="4"/>
     </row>
@@ -10530,7 +10530,7 @@
       <c r="D912" s="5"/>
       <c r="E912" s="4"/>
       <c r="F912" s="4"/>
-      <c r="G912" s="5"/>
+      <c r="G912" s="4"/>
       <c r="H912" s="4"/>
       <c r="I912" s="4"/>
     </row>
@@ -10541,7 +10541,7 @@
       <c r="D913" s="5"/>
       <c r="E913" s="4"/>
       <c r="F913" s="4"/>
-      <c r="G913" s="4"/>
+      <c r="G913" s="5"/>
       <c r="H913" s="4"/>
       <c r="I913" s="4"/>
     </row>
@@ -10585,7 +10585,7 @@
       <c r="D917" s="5"/>
       <c r="E917" s="4"/>
       <c r="F917" s="4"/>
-      <c r="G917" s="5"/>
+      <c r="G917" s="4"/>
       <c r="H917" s="4"/>
       <c r="I917" s="4"/>
     </row>
@@ -10596,7 +10596,7 @@
       <c r="D918" s="5"/>
       <c r="E918" s="4"/>
       <c r="F918" s="4"/>
-      <c r="G918" s="4"/>
+      <c r="G918" s="5"/>
       <c r="H918" s="4"/>
       <c r="I918" s="4"/>
     </row>
@@ -10618,7 +10618,7 @@
       <c r="D920" s="5"/>
       <c r="E920" s="4"/>
       <c r="F920" s="4"/>
-      <c r="G920" s="5"/>
+      <c r="G920" s="4"/>
       <c r="H920" s="4"/>
       <c r="I920" s="4"/>
     </row>
@@ -10640,7 +10640,7 @@
       <c r="D922" s="5"/>
       <c r="E922" s="4"/>
       <c r="F922" s="4"/>
-      <c r="G922" s="4"/>
+      <c r="G922" s="5"/>
       <c r="H922" s="4"/>
       <c r="I922" s="4"/>
     </row>
@@ -10651,7 +10651,7 @@
       <c r="D923" s="5"/>
       <c r="E923" s="4"/>
       <c r="F923" s="4"/>
-      <c r="G923" s="5"/>
+      <c r="G923" s="4"/>
       <c r="H923" s="4"/>
       <c r="I923" s="4"/>
     </row>
@@ -10662,7 +10662,7 @@
       <c r="D924" s="5"/>
       <c r="E924" s="4"/>
       <c r="F924" s="4"/>
-      <c r="G924" s="4"/>
+      <c r="G924" s="5"/>
       <c r="H924" s="4"/>
       <c r="I924" s="4"/>
     </row>
@@ -10728,7 +10728,7 @@
       <c r="D930" s="5"/>
       <c r="E930" s="4"/>
       <c r="F930" s="4"/>
-      <c r="G930" s="5"/>
+      <c r="G930" s="4"/>
       <c r="H930" s="4"/>
       <c r="I930" s="4"/>
     </row>
@@ -10739,7 +10739,7 @@
       <c r="D931" s="5"/>
       <c r="E931" s="4"/>
       <c r="F931" s="4"/>
-      <c r="G931" s="4"/>
+      <c r="G931" s="5"/>
       <c r="H931" s="4"/>
       <c r="I931" s="4"/>
     </row>
@@ -10871,7 +10871,7 @@
       <c r="D943" s="5"/>
       <c r="E943" s="4"/>
       <c r="F943" s="4"/>
-      <c r="G943" s="5"/>
+      <c r="G943" s="4"/>
       <c r="H943" s="4"/>
       <c r="I943" s="4"/>
     </row>
@@ -10882,7 +10882,7 @@
       <c r="D944" s="5"/>
       <c r="E944" s="4"/>
       <c r="F944" s="4"/>
-      <c r="G944" s="4"/>
+      <c r="G944" s="5"/>
       <c r="H944" s="4"/>
       <c r="I944" s="4"/>
     </row>
@@ -11014,7 +11014,7 @@
       <c r="D956" s="5"/>
       <c r="E956" s="4"/>
       <c r="F956" s="4"/>
-      <c r="G956" s="5"/>
+      <c r="G956" s="4"/>
       <c r="H956" s="4"/>
       <c r="I956" s="4"/>
     </row>
@@ -11025,7 +11025,7 @@
       <c r="D957" s="5"/>
       <c r="E957" s="4"/>
       <c r="F957" s="4"/>
-      <c r="G957" s="4"/>
+      <c r="G957" s="5"/>
       <c r="H957" s="4"/>
       <c r="I957" s="4"/>
     </row>
@@ -11102,7 +11102,7 @@
       <c r="D964" s="5"/>
       <c r="E964" s="4"/>
       <c r="F964" s="4"/>
-      <c r="G964" s="5"/>
+      <c r="G964" s="4"/>
       <c r="H964" s="4"/>
       <c r="I964" s="4"/>
     </row>
@@ -11113,7 +11113,7 @@
       <c r="D965" s="5"/>
       <c r="E965" s="4"/>
       <c r="F965" s="4"/>
-      <c r="G965" s="4"/>
+      <c r="G965" s="5"/>
       <c r="H965" s="4"/>
       <c r="I965" s="4"/>
     </row>
@@ -11146,7 +11146,7 @@
       <c r="D968" s="5"/>
       <c r="E968" s="4"/>
       <c r="F968" s="4"/>
-      <c r="G968" s="5"/>
+      <c r="G968" s="4"/>
       <c r="H968" s="4"/>
       <c r="I968" s="4"/>
     </row>
@@ -11157,7 +11157,7 @@
       <c r="D969" s="5"/>
       <c r="E969" s="4"/>
       <c r="F969" s="4"/>
-      <c r="G969" s="4"/>
+      <c r="G969" s="5"/>
       <c r="H969" s="4"/>
       <c r="I969" s="4"/>
     </row>
@@ -11256,7 +11256,7 @@
       <c r="D978" s="5"/>
       <c r="E978" s="4"/>
       <c r="F978" s="4"/>
-      <c r="G978" s="5"/>
+      <c r="G978" s="4"/>
       <c r="H978" s="4"/>
       <c r="I978" s="4"/>
     </row>
@@ -11278,7 +11278,7 @@
       <c r="D980" s="5"/>
       <c r="E980" s="4"/>
       <c r="F980" s="4"/>
-      <c r="G980" s="4"/>
+      <c r="G980" s="5"/>
       <c r="H980" s="4"/>
       <c r="I980" s="4"/>
     </row>
@@ -11311,7 +11311,7 @@
       <c r="D983" s="5"/>
       <c r="E983" s="4"/>
       <c r="F983" s="4"/>
-      <c r="G983" s="5"/>
+      <c r="G983" s="4"/>
       <c r="H983" s="4"/>
       <c r="I983" s="4"/>
     </row>
@@ -11322,7 +11322,7 @@
       <c r="D984" s="5"/>
       <c r="E984" s="4"/>
       <c r="F984" s="4"/>
-      <c r="G984" s="4"/>
+      <c r="G984" s="5"/>
       <c r="H984" s="4"/>
       <c r="I984" s="4"/>
     </row>
@@ -11333,7 +11333,7 @@
       <c r="D985" s="5"/>
       <c r="E985" s="4"/>
       <c r="F985" s="4"/>
-      <c r="G985" s="5"/>
+      <c r="G985" s="4"/>
       <c r="H985" s="4"/>
       <c r="I985" s="4"/>
     </row>
@@ -11344,7 +11344,7 @@
       <c r="D986" s="5"/>
       <c r="E986" s="4"/>
       <c r="F986" s="4"/>
-      <c r="G986" s="4"/>
+      <c r="G986" s="5"/>
       <c r="H986" s="4"/>
       <c r="I986" s="4"/>
     </row>
@@ -11377,7 +11377,7 @@
       <c r="D989" s="5"/>
       <c r="E989" s="4"/>
       <c r="F989" s="4"/>
-      <c r="G989" s="5"/>
+      <c r="G989" s="4"/>
       <c r="H989" s="4"/>
       <c r="I989" s="4"/>
     </row>
@@ -11388,7 +11388,7 @@
       <c r="D990" s="5"/>
       <c r="E990" s="4"/>
       <c r="F990" s="4"/>
-      <c r="G990" s="4"/>
+      <c r="G990" s="5"/>
       <c r="H990" s="4"/>
       <c r="I990" s="4"/>
     </row>
@@ -11432,7 +11432,7 @@
       <c r="D994" s="5"/>
       <c r="E994" s="4"/>
       <c r="F994" s="4"/>
-      <c r="G994" s="5"/>
+      <c r="G994" s="4"/>
       <c r="H994" s="4"/>
       <c r="I994" s="4"/>
     </row>
@@ -11443,7 +11443,7 @@
       <c r="D995" s="5"/>
       <c r="E995" s="4"/>
       <c r="F995" s="4"/>
-      <c r="G995" s="4"/>
+      <c r="G995" s="5"/>
       <c r="H995" s="4"/>
       <c r="I995" s="4"/>
     </row>
@@ -11454,7 +11454,7 @@
       <c r="D996" s="5"/>
       <c r="E996" s="4"/>
       <c r="F996" s="4"/>
-      <c r="G996" s="5"/>
+      <c r="G996" s="4"/>
       <c r="H996" s="4"/>
       <c r="I996" s="4"/>
     </row>
@@ -11465,7 +11465,7 @@
       <c r="D997" s="5"/>
       <c r="E997" s="4"/>
       <c r="F997" s="4"/>
-      <c r="G997" s="4"/>
+      <c r="G997" s="5"/>
       <c r="H997" s="4"/>
       <c r="I997" s="4"/>
     </row>
@@ -11498,7 +11498,7 @@
       <c r="D1000" s="5"/>
       <c r="E1000" s="4"/>
       <c r="F1000" s="4"/>
-      <c r="G1000" s="5"/>
+      <c r="G1000" s="4"/>
       <c r="H1000" s="4"/>
       <c r="I1000" s="4"/>
     </row>
@@ -11509,9 +11509,20 @@
       <c r="D1001" s="5"/>
       <c r="E1001" s="4"/>
       <c r="F1001" s="4"/>
-      <c r="G1001" s="4"/>
+      <c r="G1001" s="5"/>
       <c r="H1001" s="4"/>
       <c r="I1001" s="4"/>
+    </row>
+    <row r="1002" customFormat="false" ht="20.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1002" s="3"/>
+      <c r="B1002" s="4"/>
+      <c r="C1002" s="4"/>
+      <c r="D1002" s="5"/>
+      <c r="E1002" s="4"/>
+      <c r="F1002" s="4"/>
+      <c r="G1002" s="4"/>
+      <c r="H1002" s="4"/>
+      <c r="I1002" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>